<commit_message>
docs(mcp): bank + re-anchor — PRs #2/#3 merged, Signature persistence reconciled, MCP parked for Alpha
Per the 2026-06-04 directive: branch committed/pushed (Beta, stays off main);
PR #2 (MF-1+MF-2) and PR #3 (C1) merged after green regression gates; chosen
Signature persists LOCALLY for Alpha (IV-OS log_asset echo = Beta, reads from
the local store); next build focus is the Alpha in-app UI flow, not MCP tools.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brand-coach-mcp-planning/STATUS.xlsx
+++ b/brand-coach-mcp-planning/STATUS.xlsx
@@ -39,7 +39,7 @@
     </font>
     <font/>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -56,11 +56,6 @@
         <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -74,7 +69,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -83,9 +78,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -854,12 +846,12 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Engine EXISTS: reveal-signature edge fn (frozen no-parroting prompt, index.ts L81). Accepts conversation[] OR fields OR reviews and declines gracefully if all empty (does NOT strictly require conversation). PERSISTENCE MISSING: no signatures table/column (verified). D2 OPEN: conversation-first headless turn vs synthesize-context-bundle (latter brushes the locked no-parroting input rule -&gt; R-015).</t>
+          <t>Engine EXISTS: reveal-signature edge fn (frozen no-parroting prompt, index.ts L81). Accepts conversation[] OR fields OR reviews and declines gracefully if all empty (does NOT strictly require conversation). PERSISTENCE MISSING: no signatures table/column (verified). D2 OPEN: conversation-first headless turn vs synthesize-context-bundle (latter brushes the locked no-parroting input rule -&gt; R-015). DECISION 2026-06-04 (Matthew): chosen Signature persists LOCALLY in brand-coach for Alpha (signatures table / avatar column — local store = source of truth; in-app must NOT depend on IV-OS). IV-OS log_asset echo = Beta mechanism reading from the local store. Verified zero existing writers: no signatures migration, reveal-signature has no DB writes, MCP auto-record never touches Signatures.</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Decide D2, then pass-through reveal-signature; route any save through IV-OS log_asset (no local store).</t>
+          <t>ALPHA: build local Signature persistence (schema designed so the Beta log_asset echo reads from it without rework). D2 gates only the MCP generate_signature tool.</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -916,37 +908,37 @@
       </c>
     </row>
     <row r="13" ht="78" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>search_user_kb (diagnostic — convenience)</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>Engine EXISTS: match_document_chunks RPC (migration 20260406000000_pgvector_rag_migration.sql L53-93, pgvector ada-1536). SECURITY MF-1: SECURITY DEFINER, filters WHERE ukc.user_id = match_user_id with NO auth.uid() caller check, GRANT EXECUTE TO authenticated (confused deputy — any authenticated principal can read any owner's KB). UPDATE 2026-06-03: MF-1 confused-deputy hardened (auth.uid() guard, 4 RPCs) in PR #2 — wrap unblocked once merged.</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>Wrap the RPC; harden MF-1 inside the function before exposing.</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>Implement search_user_kb wrapping match_document_chunks. Before exposing, harden MF-1: verify inside the function that the caller is authorized (owns the id OR has an active va_grants row). Add a test that caller A cannot read caller B's KB.</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>Use a workflow: Agent A applies the MF-1 hardening migration; agent B wraps the RPC + adds the cross-owner denial test.</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1156,7 +1148,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Brand-Coach Marketing MCP - Status Workbook</t>
         </is>
@@ -1164,7 +1156,7 @@
       <c r="B1" s="3" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>Generated</t>
         </is>
@@ -1176,7 +1168,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>Canonical repo</t>
         </is>
@@ -1188,7 +1180,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Upstream dependency</t>
         </is>
@@ -1200,7 +1192,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>On Critical Path = Y</t>
         </is>
@@ -1212,19 +1204,19 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>BUILD TARGET (yellow row)</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>search_user_kb is highlighted as the FIRST post-merge build (lowest-effort wrap once PR #2 lands the MF-1 auth.uid() guard). Nothing is buildable before those merges; all critical-path components are Testing.</t>
+          <t>No highlighted build target: the MCP surface is parked at Beta. All 7 critical-path components are Testing; remaining MCP work resumes after Alpha (post-merge wraps, D2, upstream slices).</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>On Critical Path (peach rows)</t>
         </is>
@@ -1236,7 +1228,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Status values</t>
         </is>
@@ -1248,19 +1240,19 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Next Goal</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>GATED on operator actions: merge PR #2 (MF-1+MF-2) then wrap search_user_kb + build_avatar; merge PR #3 (C1) then wrap run_diagnostic; decide D2 for generate_signature. No unblocked in-repo critical-path work remains — every Y component is Testing.</t>
+          <t>RE-ANCHORED 2026-06-04 (Matthew directive): MCP work BANKED on feat/brand-coach-mcp-host (committed + pushed; stays off main until Alpha ships) and PARKED. Next build focus = Alpha in-app UI: local Signature persistence, feedback capture (feedback_events + Moment-1 modal), funnel+error instrumentation with session/user correlation key, conversation tightening. PR #2 (MF-1/MF-2 -&gt; main) and PR #3 (C1 -&gt; feat/feature-status-tracker) MERGED 2026-06-04 after a green regression gate.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Note</t>
         </is>

</xml_diff>